<commit_message>
Complete Sprint 6 final QA and acceptance
</commit_message>
<xml_diff>
--- a/dashboard_report.xlsx
+++ b/dashboard_report.xlsx
@@ -2496,12 +2496,12 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>3 Years:       30%</t>
+          <t>5 Years:       22%</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>3 Years:           26%</t>
+          <t>5 Years:           23%</t>
         </is>
       </c>
     </row>
@@ -2555,12 +2555,12 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>5 Years:       22%</t>
+          <t>3 Years:       30%</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>5 Years:           23%</t>
+          <t>3 Years:           26%</t>
         </is>
       </c>
     </row>
@@ -3501,12 +3501,12 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>3 Years:       5%</t>
+          <t>5 Years:       13%</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>3 Years:           10%</t>
+          <t>5 Years:           11%</t>
         </is>
       </c>
     </row>
@@ -3560,12 +3560,12 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>5 Years:       13%</t>
+          <t>3 Years:       5%</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>5 Years:           11%</t>
+          <t>3 Years:           10%</t>
         </is>
       </c>
     </row>
@@ -5118,12 +5118,12 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>3 Years:       17%</t>
+          <t>5 Years:       24%</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>3 Years:            9%</t>
+          <t>5 Years:            6%</t>
         </is>
       </c>
     </row>
@@ -5177,12 +5177,12 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>5 Years:       24%</t>
+          <t>3 Years:       17%</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>5 Years:            6%</t>
+          <t>3 Years:            9%</t>
         </is>
       </c>
     </row>
@@ -5661,12 +5661,12 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Years:       14%             </t>
+          <t xml:space="preserve">5 Years:       10%             </t>
         </is>
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>3 Years:            12%</t>
+          <t>5 Years:            8%</t>
         </is>
       </c>
     </row>
@@ -5720,12 +5720,12 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Years:       10%             </t>
+          <t xml:space="preserve">3 Years:       14%             </t>
         </is>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>5 Years:            8%</t>
+          <t>3 Years:            12%</t>
         </is>
       </c>
     </row>

</xml_diff>